<commit_message>
Leads: 2026-10-27 04:36 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://www.nyc1sewer.com/services</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>nyc1sewer@gmail.com</t>
@@ -554,6 +553,66 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Platinumplumbing</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>platinumplumbingvt.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.platinumplumbingvt.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>More Use</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>contact@platinumplumbingvt.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>802-777-5719</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Burlington VT</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>84</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>plumbing company Burlington VT</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-27 04:48 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -618,6 +618,62 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Marxs Roofing | Residential Roofing for the Capital Region</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>marxsroofing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://marxsroofing.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@marxsroofing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(518) 365-3230</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Schenectady NY</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>96</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>roofer Schenectady NY</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-27 14:26 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,6 @@
           <t>https://marxsroofing.com/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>info@marxsroofing.com</t>
@@ -669,6 +668,122 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Kind Roofing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>kindroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://kindroofingtx.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Story Founded</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>will@kindroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(512) 766-9755</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofing contractor Austin TX</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Roofing Contractor | Olathe, KS | 913-481-4959</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>roofing-contractor-ks.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.roofing-contractor-ks.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>capierson55@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>913-481-4959</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>86</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roofing contractor Olathe KS</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-27 14:27 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -754,7 +754,6 @@
           <t>https://www.roofing-contractor-ks.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>capierson55@yahoo.com</t>
@@ -784,6 +783,62 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OHA HVAC, Plumbing, Chimney &amp; Fireplaces</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fixmyair.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://fixmyair.com/plumbing/water-heater/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>help@fixmyair.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(571) 485-9343</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>88</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>water heater repair Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-27 14:32 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -809,7 +809,6 @@
           <t>https://fixmyair.com/plumbing/water-heater/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>help@fixmyair.com</t>
@@ -839,6 +838,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Plumbing Services | Virginia Beach, VA | Everything Plumbing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>everythingplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.everythingplumbingservices.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Hampton Roads</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>chris@everythingplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(757) 590-9992</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>plumbing company Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-27 20:35 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -903,6 +903,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Airtech Mechanical Heating, Cooling, and Plumbing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>airtechheatcool.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://airtechheatcool.com/heating/heat-pump-repair-installation/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Heat Pump</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>hvac125@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(734) 560-0582</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Livonia MI</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>heat pump installation Livonia MI</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-27 20:41 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -963,6 +963,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Archer Roofing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>archerroofingnh.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://archerroofingnh.com/roofing/concord-nh</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>nathan@archerroofingnh.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>603-931-4655</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Concord NH</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>86</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>residential roofing company Concord NH</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-27 20:48 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-27.xlsx
+++ b/output/leads_2026-10-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1023,6 +1023,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hard Roof</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>hard-roof.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://hard-roof.com/areas/concord/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Public Adjusters</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@hardroof.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>980-351-7226</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofer Concord NC</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>